<commit_message>
dash: add name column in model sheet
</commit_message>
<xml_diff>
--- a/public/files/modelo-contatos-whatsapp.xlsx
+++ b/public/files/modelo-contatos-whatsapp.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaleb\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaleb\Documents\fast-zapp\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB80D466-4BB5-4E41-85B7-3ED393AE58DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6702B88B-C825-4566-A3B2-F9A5FF84D43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contatos" sheetId="1" r:id="rId1"/>
@@ -20,21 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>11999887766</t>
   </si>
   <si>
-    <t>21987654321</t>
-  </si>
-  <si>
-    <t>31876543210</t>
-  </si>
-  <si>
-    <t>47999123456</t>
-  </si>
-  <si>
-    <t>85988776655</t>
+    <t>Lucas Alexandrino</t>
   </si>
 </sst>
 </file>
@@ -411,42 +402,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.75" customWidth="1"/>
-    <col min="2" max="2" width="13.875" customWidth="1"/>
+    <col min="1" max="1" width="28.09765625" customWidth="1"/>
+    <col min="2" max="2" width="21.69921875" customWidth="1"/>
+    <col min="3" max="3" width="13.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
+      <c r="B1" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:A5" numberStoredAsText="1"/>
+    <ignoredError sqref="B1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>